<commit_message>
fix: restore 9조 세일즈포스 data lost due to merged cells
openpyxl reads only the first cell of a merged range, so 7 of 8
members in 9조 had blank 6.24 오후 entries. Filled all with
'세일즈포스 (2호차)' to match original data. Also unmerged all
remaining merged cells in the modified Excel to prevent future
data loss.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/silicon-valley-bus-schedule.xlsx
+++ b/public/silicon-valley-bus-schedule.xlsx
@@ -2482,7 +2482,11 @@
       </c>
     </row>
     <row r="3" ht="16.05" customHeight="1" s="5">
-      <c r="A3" s="134" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B3" s="127" t="n">
         <v>2</v>
       </c>
@@ -2636,7 +2640,11 @@
       </c>
     </row>
     <row r="4" ht="16.05" customHeight="1" s="5">
-      <c r="A4" s="134" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B4" s="127" t="n">
         <v>3</v>
       </c>
@@ -2790,7 +2798,11 @@
       </c>
     </row>
     <row r="5" ht="16.05" customHeight="1" s="5">
-      <c r="A5" s="134" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B5" s="127" t="n">
         <v>4</v>
       </c>
@@ -2944,7 +2956,11 @@
       </c>
     </row>
     <row r="6" ht="16.05" customHeight="1" s="5">
-      <c r="A6" s="134" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B6" s="127" t="n">
         <v>5</v>
       </c>
@@ -3098,7 +3114,11 @@
       </c>
     </row>
     <row r="7" ht="16.05" customHeight="1" s="5">
-      <c r="A7" s="134" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B7" s="127" t="n">
         <v>6</v>
       </c>
@@ -3252,7 +3272,11 @@
       </c>
     </row>
     <row r="8" ht="16.05" customHeight="1" s="5">
-      <c r="A8" s="134" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B8" s="127" t="n">
         <v>7</v>
       </c>
@@ -3406,7 +3430,11 @@
       </c>
     </row>
     <row r="9" ht="16.05" customHeight="1" s="5">
-      <c r="A9" s="134" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B9" s="127" t="n">
         <v>8</v>
       </c>
@@ -3560,7 +3588,11 @@
       </c>
     </row>
     <row r="10" ht="16.05" customHeight="1" s="5">
-      <c r="A10" s="134" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B10" s="127" t="n">
         <v>9</v>
       </c>
@@ -3714,7 +3746,11 @@
       </c>
     </row>
     <row r="11" ht="16.05" customHeight="1" s="5">
-      <c r="A11" s="134" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B11" s="127" t="n">
         <v>10</v>
       </c>
@@ -3868,7 +3904,11 @@
       </c>
     </row>
     <row r="12" ht="16.05" customHeight="1" s="5">
-      <c r="A12" s="134" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B12" s="127" t="n">
         <v>11</v>
       </c>
@@ -4022,7 +4062,11 @@
       </c>
     </row>
     <row r="13" ht="16.05" customHeight="1" s="5">
-      <c r="A13" s="134" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B13" s="127" t="n">
         <v>12</v>
       </c>
@@ -4176,7 +4220,11 @@
       </c>
     </row>
     <row r="14" ht="16.05" customHeight="1" s="5">
-      <c r="A14" s="134" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B14" s="127" t="n">
         <v>13</v>
       </c>
@@ -4330,7 +4378,11 @@
       </c>
     </row>
     <row r="15" ht="16.05" customHeight="1" s="5">
-      <c r="A15" s="134" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B15" s="127" t="n">
         <v>14</v>
       </c>
@@ -4484,7 +4536,11 @@
       </c>
     </row>
     <row r="16" ht="16.05" customHeight="1" s="5">
-      <c r="A16" s="134" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B16" s="127" t="n">
         <v>15</v>
       </c>
@@ -4638,7 +4694,11 @@
       </c>
     </row>
     <row r="17" ht="16.05" customHeight="1" s="5">
-      <c r="A17" s="134" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B17" s="127" t="n">
         <v>16</v>
       </c>
@@ -4792,7 +4852,11 @@
       </c>
     </row>
     <row r="18" ht="16.05" customHeight="1" s="5">
-      <c r="A18" s="134" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B18" s="127" t="n">
         <v>17</v>
       </c>
@@ -4946,7 +5010,11 @@
       </c>
     </row>
     <row r="19" ht="16.05" customHeight="1" s="5">
-      <c r="A19" s="134" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B19" s="127" t="n">
         <v>18</v>
       </c>
@@ -5100,7 +5168,11 @@
       </c>
     </row>
     <row r="20" ht="16.05" customHeight="1" s="5">
-      <c r="A20" s="134" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B20" s="127" t="n">
         <v>19</v>
       </c>
@@ -5254,7 +5326,11 @@
       </c>
     </row>
     <row r="21" ht="16.05" customHeight="1" s="5">
-      <c r="A21" s="134" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B21" s="127" t="n">
         <v>20</v>
       </c>
@@ -5408,7 +5484,11 @@
       </c>
     </row>
     <row r="22" ht="16.05" customHeight="1" s="5">
-      <c r="A22" s="134" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B22" s="127" t="n">
         <v>21</v>
       </c>
@@ -5562,7 +5642,11 @@
       </c>
     </row>
     <row r="23" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A23" s="134" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B23" s="127" t="n">
         <v>22</v>
       </c>
@@ -5716,7 +5800,11 @@
       </c>
     </row>
     <row r="24" ht="16.05" customHeight="1" s="5">
-      <c r="A24" s="134" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B24" s="127" t="n">
         <v>23</v>
       </c>
@@ -5870,7 +5958,11 @@
       </c>
     </row>
     <row r="25" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A25" s="134" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B25" s="127" t="n">
         <v>24</v>
       </c>
@@ -6024,7 +6116,11 @@
       </c>
     </row>
     <row r="26" ht="16.05" customHeight="1" s="5">
-      <c r="A26" s="134" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B26" s="127" t="n">
         <v>25</v>
       </c>
@@ -6178,7 +6274,11 @@
       </c>
     </row>
     <row r="27" ht="16.05" customHeight="1" s="5">
-      <c r="A27" s="134" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B27" s="127" t="n">
         <v>26</v>
       </c>
@@ -6332,7 +6432,11 @@
       </c>
     </row>
     <row r="28" ht="16.05" customHeight="1" s="5">
-      <c r="A28" s="134" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B28" s="127" t="n">
         <v>27</v>
       </c>
@@ -6486,7 +6590,11 @@
       </c>
     </row>
     <row r="29" ht="16.05" customHeight="1" s="5">
-      <c r="A29" s="134" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B29" s="127" t="n">
         <v>28</v>
       </c>
@@ -6640,7 +6748,11 @@
       </c>
     </row>
     <row r="30" ht="16.05" customHeight="1" s="5">
-      <c r="A30" s="134" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B30" s="127" t="n">
         <v>29</v>
       </c>
@@ -6794,7 +6906,11 @@
       </c>
     </row>
     <row r="31" ht="16.05" customHeight="1" s="5">
-      <c r="A31" s="134" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B31" s="127" t="n">
         <v>30</v>
       </c>
@@ -6948,7 +7064,11 @@
       </c>
     </row>
     <row r="32" ht="16.05" customHeight="1" s="5">
-      <c r="A32" s="134" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B32" s="127" t="n">
         <v>31</v>
       </c>
@@ -7102,7 +7222,11 @@
       </c>
     </row>
     <row r="33" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A33" s="135" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B33" s="127" t="n">
         <v>32</v>
       </c>
@@ -7414,7 +7538,11 @@
       </c>
     </row>
     <row r="35" ht="16.05" customHeight="1" s="5">
-      <c r="A35" s="134" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B35" s="127" t="n">
         <v>34</v>
       </c>
@@ -7568,7 +7696,11 @@
       </c>
     </row>
     <row r="36" ht="16.05" customHeight="1" s="5">
-      <c r="A36" s="134" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B36" s="127" t="n">
         <v>35</v>
       </c>
@@ -7722,7 +7854,11 @@
       </c>
     </row>
     <row r="37" ht="16.05" customHeight="1" s="5">
-      <c r="A37" s="134" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B37" s="127" t="n">
         <v>36</v>
       </c>
@@ -7876,7 +8012,11 @@
       </c>
     </row>
     <row r="38" ht="16.05" customHeight="1" s="5">
-      <c r="A38" s="134" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B38" s="127" t="n">
         <v>37</v>
       </c>
@@ -8030,7 +8170,11 @@
       </c>
     </row>
     <row r="39" ht="16.05" customHeight="1" s="5">
-      <c r="A39" s="134" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B39" s="127" t="n">
         <v>38</v>
       </c>
@@ -8184,7 +8328,11 @@
       </c>
     </row>
     <row r="40" ht="16.05" customHeight="1" s="5">
-      <c r="A40" s="134" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B40" s="127" t="n">
         <v>39</v>
       </c>
@@ -8338,7 +8486,11 @@
       </c>
     </row>
     <row r="41" ht="16.05" customHeight="1" s="5">
-      <c r="A41" s="134" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B41" s="127" t="n">
         <v>40</v>
       </c>
@@ -8492,7 +8644,11 @@
       </c>
     </row>
     <row r="42" ht="16.05" customHeight="1" s="5">
-      <c r="A42" s="134" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B42" s="127" t="n">
         <v>41</v>
       </c>
@@ -8646,7 +8802,11 @@
       </c>
     </row>
     <row r="43" ht="16.05" customHeight="1" s="5">
-      <c r="A43" s="134" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B43" s="127" t="n">
         <v>42</v>
       </c>
@@ -8800,7 +8960,11 @@
       </c>
     </row>
     <row r="44" ht="16.05" customHeight="1" s="5">
-      <c r="A44" s="134" t="n"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B44" s="127" t="n">
         <v>43</v>
       </c>
@@ -8954,7 +9118,11 @@
       </c>
     </row>
     <row r="45" ht="16.05" customHeight="1" s="5">
-      <c r="A45" s="134" t="n"/>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B45" s="127" t="n">
         <v>44</v>
       </c>
@@ -9108,7 +9276,11 @@
       </c>
     </row>
     <row r="46" ht="16.05" customHeight="1" s="5">
-      <c r="A46" s="134" t="n"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B46" s="127" t="n">
         <v>45</v>
       </c>
@@ -9262,7 +9434,11 @@
       </c>
     </row>
     <row r="47" ht="16.05" customHeight="1" s="5">
-      <c r="A47" s="134" t="n"/>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B47" s="127" t="n">
         <v>46</v>
       </c>
@@ -9416,7 +9592,11 @@
       </c>
     </row>
     <row r="48" ht="16.05" customHeight="1" s="5">
-      <c r="A48" s="134" t="n"/>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B48" s="127" t="n">
         <v>47</v>
       </c>
@@ -9570,7 +9750,11 @@
       </c>
     </row>
     <row r="49" ht="16.05" customHeight="1" s="5">
-      <c r="A49" s="134" t="n"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B49" s="127" t="n">
         <v>48</v>
       </c>
@@ -9724,7 +9908,11 @@
       </c>
     </row>
     <row r="50" ht="16.05" customHeight="1" s="5">
-      <c r="A50" s="134" t="n"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B50" s="127" t="n">
         <v>49</v>
       </c>
@@ -9878,7 +10066,11 @@
       </c>
     </row>
     <row r="51" ht="16.05" customHeight="1" s="5">
-      <c r="A51" s="134" t="n"/>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B51" s="127" t="n">
         <v>50</v>
       </c>
@@ -10032,7 +10224,11 @@
       </c>
     </row>
     <row r="52" ht="16.05" customHeight="1" s="5">
-      <c r="A52" s="134" t="n"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B52" s="127" t="n">
         <v>51</v>
       </c>
@@ -10186,7 +10382,11 @@
       </c>
     </row>
     <row r="53" ht="16.05" customHeight="1" s="5">
-      <c r="A53" s="134" t="n"/>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B53" s="127" t="n">
         <v>52</v>
       </c>
@@ -10340,7 +10540,11 @@
       </c>
     </row>
     <row r="54" ht="16.05" customHeight="1" s="5">
-      <c r="A54" s="134" t="n"/>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B54" s="127" t="n">
         <v>53</v>
       </c>
@@ -10494,7 +10698,11 @@
       </c>
     </row>
     <row r="55" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A55" s="134" t="n"/>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B55" s="127" t="n">
         <v>54</v>
       </c>
@@ -10648,7 +10856,11 @@
       </c>
     </row>
     <row r="56" ht="16.05" customHeight="1" s="5">
-      <c r="A56" s="134" t="n"/>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B56" s="127" t="n">
         <v>55</v>
       </c>
@@ -10802,7 +11014,11 @@
       </c>
     </row>
     <row r="57" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A57" s="134" t="n"/>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B57" s="127" t="n">
         <v>56</v>
       </c>
@@ -10956,7 +11172,11 @@
       </c>
     </row>
     <row r="58" ht="16.05" customHeight="1" s="5">
-      <c r="A58" s="134" t="n"/>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B58" s="127" t="n">
         <v>57</v>
       </c>
@@ -11110,7 +11330,11 @@
       </c>
     </row>
     <row r="59" ht="16.05" customHeight="1" s="5">
-      <c r="A59" s="134" t="n"/>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B59" s="127" t="n">
         <v>58</v>
       </c>
@@ -11264,7 +11488,11 @@
       </c>
     </row>
     <row r="60" ht="16.05" customHeight="1" s="5">
-      <c r="A60" s="134" t="n"/>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B60" s="127" t="n">
         <v>59</v>
       </c>
@@ -11418,7 +11646,11 @@
       </c>
     </row>
     <row r="61" ht="16.05" customHeight="1" s="5">
-      <c r="A61" s="134" t="n"/>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B61" s="127" t="n">
         <v>60</v>
       </c>
@@ -11572,7 +11804,11 @@
       </c>
     </row>
     <row r="62" ht="16.05" customHeight="1" s="5">
-      <c r="A62" s="134" t="n"/>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B62" s="127" t="n">
         <v>61</v>
       </c>
@@ -11726,7 +11962,11 @@
       </c>
     </row>
     <row r="63" ht="16.05" customHeight="1" s="5">
-      <c r="A63" s="134" t="n"/>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B63" s="127" t="n">
         <v>62</v>
       </c>
@@ -11880,7 +12120,11 @@
       </c>
     </row>
     <row r="64" ht="16.05" customHeight="1" s="5">
-      <c r="A64" s="134" t="n"/>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B64" s="127" t="n">
         <v>63</v>
       </c>
@@ -12034,7 +12278,11 @@
       </c>
     </row>
     <row r="65" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A65" s="135" t="n"/>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B65" s="127" t="n">
         <v>64</v>
       </c>
@@ -12346,7 +12594,11 @@
       </c>
     </row>
     <row r="67" ht="16.05" customHeight="1" s="5">
-      <c r="A67" s="134" t="n"/>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B67" s="127" t="n">
         <v>66</v>
       </c>
@@ -12500,7 +12752,11 @@
       </c>
     </row>
     <row r="68" ht="16.05" customHeight="1" s="5">
-      <c r="A68" s="134" t="n"/>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B68" s="127" t="n">
         <v>67</v>
       </c>
@@ -12654,7 +12910,11 @@
       </c>
     </row>
     <row r="69" ht="16.05" customHeight="1" s="5">
-      <c r="A69" s="134" t="n"/>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B69" s="127" t="n">
         <v>68</v>
       </c>
@@ -12808,7 +13068,11 @@
       </c>
     </row>
     <row r="70" ht="16.05" customHeight="1" s="5">
-      <c r="A70" s="134" t="n"/>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B70" s="127" t="n">
         <v>69</v>
       </c>
@@ -12962,7 +13226,11 @@
       </c>
     </row>
     <row r="71" ht="16.05" customHeight="1" s="5">
-      <c r="A71" s="134" t="n"/>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B71" s="127" t="n">
         <v>70</v>
       </c>
@@ -13116,7 +13384,11 @@
       </c>
     </row>
     <row r="72" ht="16.05" customHeight="1" s="5">
-      <c r="A72" s="134" t="n"/>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B72" s="127" t="n">
         <v>71</v>
       </c>
@@ -13270,7 +13542,11 @@
       </c>
     </row>
     <row r="73" ht="16.05" customHeight="1" s="5">
-      <c r="A73" s="134" t="n"/>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B73" s="127" t="n">
         <v>72</v>
       </c>
@@ -13424,7 +13700,11 @@
       </c>
     </row>
     <row r="74" ht="18" customHeight="1" s="5">
-      <c r="A74" s="134" t="n"/>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B74" s="127" t="n">
         <v>73</v>
       </c>
@@ -13578,7 +13858,11 @@
       </c>
     </row>
     <row r="75" ht="18" customHeight="1" s="5">
-      <c r="A75" s="134" t="n"/>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B75" s="127" t="n">
         <v>74</v>
       </c>
@@ -13732,7 +14016,11 @@
       </c>
     </row>
     <row r="76" ht="18" customHeight="1" s="5">
-      <c r="A76" s="134" t="n"/>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B76" s="127" t="n">
         <v>75</v>
       </c>
@@ -13886,7 +14174,11 @@
       </c>
     </row>
     <row r="77" ht="18" customHeight="1" s="5">
-      <c r="A77" s="134" t="n"/>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B77" s="127" t="n">
         <v>76</v>
       </c>
@@ -14040,7 +14332,11 @@
       </c>
     </row>
     <row r="78" ht="18" customHeight="1" s="5">
-      <c r="A78" s="134" t="n"/>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B78" s="127" t="n">
         <v>77</v>
       </c>
@@ -14194,7 +14490,11 @@
       </c>
     </row>
     <row r="79" ht="18" customHeight="1" s="5">
-      <c r="A79" s="134" t="n"/>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B79" s="127" t="n">
         <v>78</v>
       </c>
@@ -14348,7 +14648,11 @@
       </c>
     </row>
     <row r="80" ht="18" customHeight="1" s="5">
-      <c r="A80" s="134" t="n"/>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B80" s="127" t="n">
         <v>79</v>
       </c>
@@ -14502,7 +14806,11 @@
       </c>
     </row>
     <row r="81" ht="18" customHeight="1" s="5">
-      <c r="A81" s="134" t="n"/>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B81" s="127" t="n">
         <v>80</v>
       </c>
@@ -14656,7 +14964,11 @@
       </c>
     </row>
     <row r="82" ht="16.05" customHeight="1" s="5">
-      <c r="A82" s="134" t="n"/>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B82" s="127" t="n">
         <v>81</v>
       </c>
@@ -14810,7 +15122,11 @@
       </c>
     </row>
     <row r="83" ht="16.05" customHeight="1" s="5">
-      <c r="A83" s="134" t="n"/>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B83" s="127" t="n">
         <v>82</v>
       </c>
@@ -14842,7 +15158,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I83" s="134" t="n"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J83" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -14960,7 +15280,11 @@
       </c>
     </row>
     <row r="84" ht="16.05" customHeight="1" s="5">
-      <c r="A84" s="134" t="n"/>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B84" s="127" t="n">
         <v>83</v>
       </c>
@@ -14992,7 +15316,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I84" s="134" t="n"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J84" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15110,7 +15438,11 @@
       </c>
     </row>
     <row r="85" ht="16.05" customHeight="1" s="5">
-      <c r="A85" s="134" t="n"/>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B85" s="127" t="n">
         <v>84</v>
       </c>
@@ -15142,7 +15474,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I85" s="134" t="n"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J85" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15260,7 +15596,11 @@
       </c>
     </row>
     <row r="86" ht="16.05" customHeight="1" s="5">
-      <c r="A86" s="134" t="n"/>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B86" s="127" t="n">
         <v>85</v>
       </c>
@@ -15292,7 +15632,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I86" s="134" t="n"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J86" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15410,7 +15754,11 @@
       </c>
     </row>
     <row r="87" ht="16.05" customHeight="1" s="5">
-      <c r="A87" s="134" t="n"/>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B87" s="127" t="n">
         <v>86</v>
       </c>
@@ -15442,7 +15790,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I87" s="134" t="n"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J87" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15560,7 +15912,11 @@
       </c>
     </row>
     <row r="88" ht="16.05" customHeight="1" s="5">
-      <c r="A88" s="134" t="n"/>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B88" s="127" t="n">
         <v>87</v>
       </c>
@@ -15592,7 +15948,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I88" s="134" t="n"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J88" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15710,7 +16070,11 @@
       </c>
     </row>
     <row r="89" ht="16.05" customHeight="1" s="5">
-      <c r="A89" s="134" t="n"/>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B89" s="127" t="n">
         <v>88</v>
       </c>
@@ -15742,7 +16106,11 @@
           <t>쌀국수 (3호차)</t>
         </is>
       </c>
-      <c r="I89" s="138" t="n"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>세일즈포스 (2호차)</t>
+        </is>
+      </c>
       <c r="J89" s="15" t="inlineStr">
         <is>
           <t>인앤아웃 (2호차)</t>
@@ -15860,7 +16228,11 @@
       </c>
     </row>
     <row r="90" ht="16.05" customHeight="1" s="5">
-      <c r="A90" s="134" t="n"/>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B90" s="127" t="n">
         <v>89</v>
       </c>
@@ -16014,7 +16386,11 @@
       </c>
     </row>
     <row r="91" ht="16.05" customHeight="1" s="5">
-      <c r="A91" s="134" t="n"/>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B91" s="127" t="n">
         <v>90</v>
       </c>
@@ -16168,7 +16544,11 @@
       </c>
     </row>
     <row r="92" ht="16.05" customHeight="1" s="5">
-      <c r="A92" s="134" t="n"/>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B92" s="127" t="n">
         <v>91</v>
       </c>
@@ -16322,7 +16702,11 @@
       </c>
     </row>
     <row r="93" ht="16.05" customHeight="1" s="5">
-      <c r="A93" s="134" t="n"/>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B93" s="127" t="n">
         <v>92</v>
       </c>
@@ -16476,7 +16860,11 @@
       </c>
     </row>
     <row r="94" ht="16.05" customHeight="1" s="5">
-      <c r="A94" s="134" t="n"/>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B94" s="127" t="n">
         <v>93</v>
       </c>
@@ -16630,7 +17018,11 @@
       </c>
     </row>
     <row r="95" ht="16.05" customHeight="1" s="5">
-      <c r="A95" s="134" t="n"/>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B95" s="127" t="n">
         <v>94</v>
       </c>
@@ -16784,7 +17176,11 @@
       </c>
     </row>
     <row r="96" ht="16.05" customHeight="1" s="5">
-      <c r="A96" s="134" t="n"/>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B96" s="127" t="n">
         <v>95</v>
       </c>
@@ -16938,7 +17334,11 @@
       </c>
     </row>
     <row r="97" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A97" s="135" t="n"/>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B97" s="83" t="n">
         <v>96</v>
       </c>
@@ -17250,7 +17650,11 @@
       </c>
     </row>
     <row r="99" ht="16.05" customHeight="1" s="5">
-      <c r="A99" s="134" t="n"/>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B99" s="127" t="n">
         <v>98</v>
       </c>
@@ -17404,7 +17808,11 @@
       </c>
     </row>
     <row r="100" ht="16.05" customHeight="1" s="5">
-      <c r="A100" s="134" t="n"/>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B100" s="127" t="n">
         <v>99</v>
       </c>
@@ -17558,7 +17966,11 @@
       </c>
     </row>
     <row r="101" ht="16.05" customHeight="1" s="5">
-      <c r="A101" s="134" t="n"/>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B101" s="127" t="n">
         <v>100</v>
       </c>
@@ -17712,7 +18124,11 @@
       </c>
     </row>
     <row r="102" ht="16.05" customHeight="1" s="5">
-      <c r="A102" s="134" t="n"/>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B102" s="127" t="n">
         <v>101</v>
       </c>
@@ -17866,7 +18282,11 @@
       </c>
     </row>
     <row r="103" ht="16.05" customHeight="1" s="5">
-      <c r="A103" s="134" t="n"/>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B103" s="127" t="n">
         <v>102</v>
       </c>
@@ -18020,7 +18440,11 @@
       </c>
     </row>
     <row r="104" ht="16.05" customHeight="1" s="5">
-      <c r="A104" s="134" t="n"/>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B104" s="127" t="n">
         <v>103</v>
       </c>
@@ -18174,7 +18598,11 @@
       </c>
     </row>
     <row r="105" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A105" s="134" t="n"/>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B105" s="127" t="n">
         <v>104</v>
       </c>
@@ -18328,7 +18756,11 @@
       </c>
     </row>
     <row r="106" ht="16.05" customHeight="1" s="5">
-      <c r="A106" s="134" t="n"/>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B106" s="127" t="n">
         <v>105</v>
       </c>
@@ -18482,7 +18914,11 @@
       </c>
     </row>
     <row r="107" ht="16.05" customHeight="1" s="5">
-      <c r="A107" s="134" t="n"/>
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B107" s="127" t="n">
         <v>106</v>
       </c>
@@ -18636,7 +19072,11 @@
       </c>
     </row>
     <row r="108" ht="16.05" customHeight="1" s="5">
-      <c r="A108" s="134" t="n"/>
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B108" s="127" t="n">
         <v>107</v>
       </c>
@@ -18790,7 +19230,11 @@
       </c>
     </row>
     <row r="109" ht="16.05" customHeight="1" s="5">
-      <c r="A109" s="134" t="n"/>
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B109" s="127" t="n">
         <v>108</v>
       </c>
@@ -18944,7 +19388,11 @@
       </c>
     </row>
     <row r="110" ht="16.05" customHeight="1" s="5">
-      <c r="A110" s="134" t="n"/>
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B110" s="127" t="n">
         <v>109</v>
       </c>
@@ -19098,7 +19546,11 @@
       </c>
     </row>
     <row r="111" ht="16.05" customHeight="1" s="5">
-      <c r="A111" s="134" t="n"/>
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B111" s="127" t="n">
         <v>110</v>
       </c>
@@ -19252,7 +19704,11 @@
       </c>
     </row>
     <row r="112" ht="16.05" customHeight="1" s="5">
-      <c r="A112" s="134" t="n"/>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B112" s="127" t="n">
         <v>111</v>
       </c>
@@ -19406,7 +19862,11 @@
       </c>
     </row>
     <row r="113" ht="16.05" customHeight="1" s="5">
-      <c r="A113" s="134" t="n"/>
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B113" s="127" t="n">
         <v>112</v>
       </c>
@@ -19560,7 +20020,11 @@
       </c>
     </row>
     <row r="114" ht="16.05" customHeight="1" s="5">
-      <c r="A114" s="134" t="n"/>
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B114" s="127" t="n">
         <v>113</v>
       </c>
@@ -19714,7 +20178,11 @@
       </c>
     </row>
     <row r="115" ht="16.05" customHeight="1" s="5">
-      <c r="A115" s="134" t="n"/>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B115" s="127" t="n">
         <v>114</v>
       </c>
@@ -19868,7 +20336,11 @@
       </c>
     </row>
     <row r="116" ht="16.05" customHeight="1" s="5">
-      <c r="A116" s="134" t="n"/>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B116" s="127" t="n">
         <v>115</v>
       </c>
@@ -20022,7 +20494,11 @@
       </c>
     </row>
     <row r="117" ht="16.05" customHeight="1" s="5">
-      <c r="A117" s="134" t="n"/>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B117" s="127" t="n">
         <v>116</v>
       </c>
@@ -20176,7 +20652,11 @@
       </c>
     </row>
     <row r="118" ht="16.05" customHeight="1" s="5">
-      <c r="A118" s="134" t="n"/>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B118" s="127" t="n">
         <v>117</v>
       </c>
@@ -20330,7 +20810,11 @@
       </c>
     </row>
     <row r="119" ht="16.05" customHeight="1" s="5">
-      <c r="A119" s="134" t="n"/>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B119" s="127" t="n">
         <v>118</v>
       </c>
@@ -20484,7 +20968,11 @@
       </c>
     </row>
     <row r="120" ht="16.05" customHeight="1" s="5">
-      <c r="A120" s="134" t="n"/>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B120" s="127" t="n">
         <v>119</v>
       </c>
@@ -20638,7 +21126,11 @@
       </c>
     </row>
     <row r="121" ht="16.05" customHeight="1" s="5">
-      <c r="A121" s="134" t="n"/>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B121" s="127" t="n">
         <v>120</v>
       </c>
@@ -20792,7 +21284,11 @@
       </c>
     </row>
     <row r="122" ht="16.05" customHeight="1" s="5">
-      <c r="A122" s="134" t="n"/>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B122" s="127" t="n">
         <v>121</v>
       </c>
@@ -20946,7 +21442,11 @@
       </c>
     </row>
     <row r="123" ht="16.05" customHeight="1" s="5">
-      <c r="A123" s="134" t="n"/>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B123" s="127" t="n">
         <v>122</v>
       </c>
@@ -21100,7 +21600,11 @@
       </c>
     </row>
     <row r="124" ht="16.05" customHeight="1" s="5">
-      <c r="A124" s="134" t="n"/>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B124" s="127" t="n">
         <v>123</v>
       </c>
@@ -21254,7 +21758,11 @@
       </c>
     </row>
     <row r="125" ht="16.05" customHeight="1" s="5">
-      <c r="A125" s="134" t="n"/>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B125" s="127" t="n">
         <v>124</v>
       </c>
@@ -21408,7 +21916,11 @@
       </c>
     </row>
     <row r="126" ht="16.05" customHeight="1" s="5">
-      <c r="A126" s="134" t="n"/>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B126" s="127" t="n">
         <v>125</v>
       </c>
@@ -21562,7 +22074,11 @@
       </c>
     </row>
     <row r="127" ht="16.05" customHeight="1" s="5">
-      <c r="A127" s="134" t="n"/>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B127" s="127" t="n">
         <v>126</v>
       </c>
@@ -21716,7 +22232,11 @@
       </c>
     </row>
     <row r="128" ht="16.05" customHeight="1" s="5">
-      <c r="A128" s="134" t="n"/>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B128" s="127" t="n">
         <v>127</v>
       </c>
@@ -21870,7 +22390,11 @@
       </c>
     </row>
     <row r="129" ht="16.05" customHeight="1" s="5">
-      <c r="A129" s="134" t="n"/>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B129" s="127" t="n">
         <v>128</v>
       </c>
@@ -22024,7 +22548,11 @@
       </c>
     </row>
     <row r="130" ht="16.05" customHeight="1" s="5" thickBot="1">
-      <c r="A130" s="135" t="n"/>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B130" s="114" t="n">
         <v>129</v>
       </c>
@@ -22424,7 +22952,11 @@
       </c>
     </row>
     <row r="133" ht="16.05" customHeight="1" s="5">
-      <c r="A133" s="134" t="n"/>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B133" s="127" t="n">
         <v>131</v>
       </c>
@@ -22580,7 +23112,11 @@
       </c>
     </row>
     <row r="134" ht="16.05" customHeight="1" s="5">
-      <c r="A134" s="138" t="n"/>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1호차</t>
+        </is>
+      </c>
       <c r="B134" s="127" t="n">
         <v>132</v>
       </c>
@@ -22896,7 +23432,11 @@
       </c>
     </row>
     <row r="136" ht="16.05" customHeight="1" s="5">
-      <c r="A136" s="134" t="n"/>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B136" s="127" t="n">
         <v>134</v>
       </c>
@@ -23052,7 +23592,11 @@
       </c>
     </row>
     <row r="137" ht="16.05" customHeight="1" s="5">
-      <c r="A137" s="138" t="n"/>
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2호차</t>
+        </is>
+      </c>
       <c r="B137" s="127" t="n">
         <v>135</v>
       </c>
@@ -23368,7 +23912,11 @@
       </c>
     </row>
     <row r="139" ht="16.05" customHeight="1" s="5">
-      <c r="A139" s="138" t="n"/>
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>3호차</t>
+        </is>
+      </c>
       <c r="B139" s="127" t="n">
         <v>137</v>
       </c>
@@ -23684,7 +24232,11 @@
       </c>
     </row>
     <row r="141" ht="16.05" customHeight="1" s="5">
-      <c r="A141" s="138" t="n"/>
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B141" s="127" t="n">
         <v>139</v>
       </c>
@@ -24558,7 +25110,11 @@
       </c>
     </row>
     <row r="147" ht="16.05" customHeight="1" s="5">
-      <c r="A147" s="126" t="n"/>
+      <c r="A147" s="126" t="inlineStr">
+        <is>
+          <t>4호차</t>
+        </is>
+      </c>
       <c r="B147" s="127" t="n">
         <v>144</v>
       </c>
@@ -24830,17 +25386,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A132:A134"/>
-    <mergeCell ref="A66:A97"/>
-    <mergeCell ref="A135:A137"/>
-    <mergeCell ref="A140:A141"/>
-    <mergeCell ref="A2:A33"/>
-    <mergeCell ref="A34:A65"/>
-    <mergeCell ref="I82:I89"/>
-    <mergeCell ref="A98:A130"/>
-    <mergeCell ref="A138:A139"/>
-  </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="portrait" scale="32"/>
   <headerFooter>

</xml_diff>